<commit_message>
AI Vision feature Implementation
</commit_message>
<xml_diff>
--- a/test_cases/test_results.xlsx
+++ b/test_cases/test_results.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="540" windowWidth="23655" windowHeight="9915" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -45,8 +45,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -519,7 +522,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
         </is>
       </c>
     </row>
@@ -564,7 +567,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
         </is>
       </c>
     </row>
@@ -613,11 +616,11 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="405" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>TC-004</t>
@@ -633,7 +636,7 @@
           <t>Happy Path</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>OPEN: /
 FILL: city-input = New York
@@ -659,8 +662,8 @@
 CLICK: confirm-booking-button
 WAIT_FOR: booking-confirmation
 OPEN: /bookings
-WAIT_FOR: booking-card-1
-ASSERT_VISIBLE: booking-card-1
+WAIT_FOR: bookings-page
+ASSERT_VISIBLE: bookings-page
 SCREENSHOT: TC-004_step-26_success</t>
         </is>
       </c>
@@ -671,12 +674,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
         </is>
       </c>
     </row>
@@ -737,7 +740,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
         </is>
       </c>
     </row>
@@ -798,7 +801,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
         </is>
       </c>
     </row>
@@ -859,7 +862,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
         </is>
       </c>
     </row>
@@ -920,7 +923,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
         </is>
       </c>
     </row>
@@ -981,7 +984,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1045,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1106,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[UNCERTAIN] (PASS:1 FAIL:0 UNCERTAIN:1) Deterministic checks passed; AI was UNCERTAIN on 1 checkpoint(s).</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1167,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) Deterministic checks passed; AI was UNCERTAIN on 2 checkpoint(s).</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1228,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) Deterministic checks passed; AI was UNCERTAIN on 2 checkpoint(s).</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1289,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) Deterministic checks passed; AI was UNCERTAIN on 2 checkpoint(s).</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1350,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>AI verification not implemented yet (Part 3 Stage 2).</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) Deterministic checks passed; AI was UNCERTAIN on 2 checkpoint(s).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EXCEL UPDATE + CONCURRENCY Feature
</commit_message>
<xml_diff>
--- a/test_cases/test_results.xlsx
+++ b/test_cases/test_results.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="540" windowWidth="23655" windowHeight="9915" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -522,7 +522,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The booking reference element visibly contains the text 'BK-387717', which includes the required 'BK-' prefix.</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The first room card for 'Grand Hotel' is clearly visible in the search results.</t>
         </is>
       </c>
     </row>
@@ -616,11 +616,11 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="405" customHeight="1">
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The room price of $150 per night is clearly visible in a blue container on the right side of the page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="21" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>TC-004</t>
@@ -679,7 +679,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The 'My Bookings' page is clearly visible, displaying a confirmed booking for Grand Hotel.</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The validation error message 'First name is required.' is clearly visible below the First Name input field.</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The validation error message 'Last name is required.' is clearly visible below the Last Name input field.</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
+          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The validation error message 'Please enter a valid email address.' is clearly visible below the email field.</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
+          <t>[UNCERTAIN] (PASS:1 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) All 2 AI visual checkpoint(s) passed.</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:1 FAIL:0 UNCERTAIN:1) Deterministic checks passed; AI was UNCERTAIN on 1 checkpoint(s).</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) Deterministic checks passed; AI was UNCERTAIN on 2 checkpoint(s).</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) Deterministic checks passed; AI was UNCERTAIN on 2 checkpoint(s).</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) Deterministic checks passed; AI was UNCERTAIN on 2 checkpoint(s).</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) Deterministic checks passed; AI was UNCERTAIN on 2 checkpoint(s).</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>

</xml_diff>